<commit_message>
Added remaining length to the end of the generated cut list
</commit_message>
<xml_diff>
--- a/CutlistTestSheet_Cutlist_.xlsx
+++ b/CutlistTestSheet_Cutlist_.xlsx
@@ -38,6 +38,9 @@
   </x:si>
   <x:si>
     <x:t>Ca1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Drop(in):</x:t>
   </x:si>
   <x:si>
     <x:t>Stick 2</x:t>
@@ -530,7 +533,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:Z47"/>
+  <x:dimension ref="A1:Z54"/>
   <x:sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="12.424911" style="0" customWidth="1"/>
@@ -598,31 +601,31 @@
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:26">
-      <x:c r="A9" s="1" t="s">
+    <x:row r="8" spans="1:26">
+      <x:c r="A8" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B8" s="1">
+        <x:v>0.6875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:26">
+      <x:c r="A10" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:26">
-      <x:c r="A10" s="3" t="s">
+      <x:c r="B10" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:26">
+      <x:c r="A11" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B10" s="3">
+      <x:c r="B11" s="3">
         <x:v>53.375</x:v>
       </x:c>
-      <x:c r="C10" s="4" t="s">
+      <x:c r="C11" s="4" t="s">
         <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:26">
-      <x:c r="A11" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="2">
-        <x:v>47.1875</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:26">
@@ -630,88 +633,88 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="2">
+        <x:v>47.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:26">
+      <x:c r="A13" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B13" s="2">
         <x:v>33.25</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:26">
-      <x:c r="A13" s="5" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B13" s="5">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="s">
+    <x:row r="14" spans="1:26">
+      <x:c r="A14" s="5" t="s">
         <x:v>12</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" spans="1:26">
-      <x:c r="A14" s="2" t="s">
+      <x:c r="B14" s="5">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B14" s="2">
+    </x:row>
+    <x:row r="15" spans="1:26">
+      <x:c r="A15" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" s="2">
         <x:v>30.4375</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:26">
-      <x:c r="A15" s="5" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B15" s="5">
-        <x:v>28.4375</x:v>
-      </x:c>
-      <x:c r="C15" s="6" t="s">
-        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:26">
       <x:c r="A16" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B16" s="5">
+        <x:v>28.4375</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:26">
+      <x:c r="A17" s="5" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B17" s="5">
         <x:v>11.4375</x:v>
       </x:c>
-      <x:c r="C16" s="6" t="s">
-        <x:v>15</x:v>
+      <x:c r="C17" s="6" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:26">
       <x:c r="A18" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B18" s="1">
+        <x:v>2.5625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:26">
+      <x:c r="A20" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B18" s="1" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:26">
-      <x:c r="A19" s="2" t="s">
+      <x:c r="B20" s="1" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="B19" s="2">
-        <x:v>24.4375</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:26">
-      <x:c r="A20" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B20" s="2">
-        <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:26">
       <x:c r="A21" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B21" s="2">
-        <x:v>5</x:v>
+        <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:26">
       <x:c r="A22" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B22" s="2">
-        <x:v>5</x:v>
+        <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:26">
@@ -746,73 +749,73 @@
         <x:v>5</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" spans="1:26">
+      <x:c r="A27" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B27" s="2">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
     <x:row r="28" spans="1:26">
-      <x:c r="A28" s="1" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B28" s="1" t="s">
+      <x:c r="A28" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B28" s="2">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:26">
+      <x:c r="A29" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B29" s="1">
+        <x:v>159.625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:26">
+      <x:c r="A31" s="1" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" spans="1:26">
-      <x:c r="A29" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B29" s="2">
+    <x:row r="32" spans="1:26">
+      <x:c r="A32" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B32" s="2">
         <x:v>20.6875</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" spans="1:26">
-      <x:c r="A30" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B30" s="2">
-        <x:v>20.6875</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" spans="1:26">
-      <x:c r="A32" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B32" s="1" t="s">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:26">
       <x:c r="A33" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B33" s="2">
+        <x:v>20.6875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:26">
+      <x:c r="A34" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B34" s="1">
+        <x:v>246.25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:26">
+      <x:c r="A36" s="1" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B33" s="2">
-        <x:v>32</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" spans="1:26">
-      <x:c r="A34" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B34" s="2">
-        <x:v>32</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" spans="1:26">
-      <x:c r="A35" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B35" s="2">
-        <x:v>32</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" spans="1:26">
-      <x:c r="A36" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B36" s="2">
-        <x:v>32</x:v>
+      <x:c r="B36" s="1" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:26">
       <x:c r="A37" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B37" s="2">
         <x:v>32</x:v>
@@ -820,7 +823,7 @@
     </x:row>
     <x:row r="38" spans="1:26">
       <x:c r="A38" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B38" s="2">
         <x:v>32</x:v>
@@ -828,7 +831,7 @@
     </x:row>
     <x:row r="39" spans="1:26">
       <x:c r="A39" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B39" s="2">
         <x:v>32</x:v>
@@ -836,23 +839,31 @@
     </x:row>
     <x:row r="40" spans="1:26">
       <x:c r="A40" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B40" s="2">
         <x:v>32</x:v>
       </x:c>
     </x:row>
+    <x:row r="41" spans="1:26">
+      <x:c r="A41" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B41" s="2">
+        <x:v>32</x:v>
+      </x:c>
+    </x:row>
     <x:row r="42" spans="1:26">
-      <x:c r="A42" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B42" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A42" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B42" s="2">
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:26">
       <x:c r="A43" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B43" s="2">
         <x:v>32</x:v>
@@ -860,29 +871,77 @@
     </x:row>
     <x:row r="44" spans="1:26">
       <x:c r="A44" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B44" s="2">
+        <x:v>32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:26">
+      <x:c r="A45" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B45" s="1">
+        <x:v>30.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:26">
+      <x:c r="A47" s="1" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B44" s="2">
-        <x:v>32</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" spans="1:26">
-      <x:c r="A46" s="1" t="s">
+      <x:c r="B47" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:26">
+      <x:c r="A48" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B46" s="1" t="s">
+      <x:c r="B48" s="2">
+        <x:v>32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:26">
+      <x:c r="A49" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B49" s="2">
+        <x:v>32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:26">
+      <x:c r="A50" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B50" s="1">
+        <x:v>223.625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" spans="1:26">
+      <x:c r="A52" s="1" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B52" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" spans="1:26">
-      <x:c r="A47" s="5" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B47" s="5">
+    <x:row r="53" spans="1:26">
+      <x:c r="A53" s="5" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B53" s="5">
         <x:v>11.4375</x:v>
       </x:c>
-      <x:c r="C47" s="6" t="s">
-        <x:v>15</x:v>
+      <x:c r="C53" s="6" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" spans="1:26">
+      <x:c r="A54" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B54" s="1">
+        <x:v>228.375</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -891,7 +950,7 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" verticalDpi="300"/>
   <x:headerFooter/>
   <x:rowBreaks count="1" manualBreakCount="1">
-    <x:brk id="31" max="1048576" man="1"/>
+    <x:brk id="35" max="1048576" man="1"/>
   </x:rowBreaks>
   <x:tableParts count="0"/>
 </x:worksheet>

</xml_diff>